<commit_message>
test: add test data creation script and conversation flow test
Created comprehensive test data:
- MySQL: 5 categories, 8 products, 10 orders
- Excel: 5 customers with VIP levels
- Self-referencing links (Category.parent)
- Cross-datasource links (Order → Customer in Excel)

Test scenarios:
1. Basic queries (search iPhone)
2. Reverse navigation (get product orders)
3. Cross-datasource links (VIP customer orders)
4. Multi-hop navigation (Category → Product → Order → Customer)
5. Aggregation (sales by category)
6. Self-referencing links (category hierarchy)

Ready for frontend testing!

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/test_customers.xlsx
+++ b/backend/test_customers.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,16 @@
           <t>vip_level</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -461,6 +471,16 @@
           <t>金卡</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>13800138001</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -478,6 +498,16 @@
           <t>银卡</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>13800138002</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -492,7 +522,71 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>金卡</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>13800138003</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>深圳</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>赵六</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>普通</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>13800138004</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>钱七</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>银卡</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>13800138005</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>杭州</t>
         </is>
       </c>
     </row>

</xml_diff>